<commit_message>
Update roster and shift plans CSV and Excel files; modify bulk upload form links for meal plans
</commit_message>
<xml_diff>
--- a/public/assets/excel/roster_plans.xlsx
+++ b/public/assets/excel/roster_plans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo LOQ\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3F6F45-DC49-4172-98DA-22FF6B0251D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083FF6E9-22B4-4B08-B46F-495AD89FCA66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,91 +20,106 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
-  <si>
-    <t>Short Name</t>
-  </si>
-  <si>
-    <t>Swapping</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>First Shift Name</t>
-  </si>
-  <si>
-    <t>Second Shift Name</t>
-  </si>
-  <si>
-    <t>Alpha Team</t>
-  </si>
-  <si>
-    <t>Beta Squad</t>
-  </si>
-  <si>
-    <t>Gamma Unit</t>
-  </si>
-  <si>
-    <t>Delta Crew</t>
-  </si>
-  <si>
-    <t>Epsilon Group</t>
-  </si>
-  <si>
-    <t>A-Team</t>
-  </si>
-  <si>
-    <t>Beta</t>
-  </si>
-  <si>
-    <t>Delta</t>
-  </si>
-  <si>
-    <t>Eps</t>
-  </si>
-  <si>
-    <t>Primary roster for project Alpha.</t>
-  </si>
-  <si>
-    <t>Backup roster for Beta operations.</t>
-  </si>
-  <si>
-    <t>Ad-hoc tasks and on-call staff.</t>
-  </si>
-  <si>
-    <t>Day-shift focused crew.</t>
-  </si>
-  <si>
-    <t>Flexible roster for overflow.</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Inactive</t>
-  </si>
-  <si>
-    <t>Morning 1</t>
-  </si>
-  <si>
-    <t>Morning 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Name</t>
-  </si>
-  <si>
-    <t>Gamma</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+  <si>
+    <t>short_name</t>
+  </si>
+  <si>
+    <t>swapping</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>first_shift_name</t>
+  </si>
+  <si>
+    <t>second_shift_name</t>
+  </si>
+  <si>
+    <t>Roster Plan Alpha</t>
+  </si>
+  <si>
+    <t>Roster Plan Bravo</t>
+  </si>
+  <si>
+    <t>Roster Plan Charlie</t>
+  </si>
+  <si>
+    <t>Roster Plan Delta</t>
+  </si>
+  <si>
+    <t>Roster Plan Echo</t>
+  </si>
+  <si>
+    <t>RP-A</t>
+  </si>
+  <si>
+    <t>RP-B</t>
+  </si>
+  <si>
+    <t>RP-C</t>
+  </si>
+  <si>
+    <t>RP-D</t>
+  </si>
+  <si>
+    <t>RP-E</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Main morning + flexible overlap</t>
+  </si>
+  <si>
+    <t>Split morning shifts for coverage</t>
+  </si>
+  <si>
+    <t>Extended morning rotation</t>
+  </si>
+  <si>
+    <t>Half-day + backup</t>
+  </si>
+  <si>
+    <t>Flexible mix for part-timers</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>inactive</t>
+  </si>
+  <si>
+    <t>Morning Shift A</t>
+  </si>
+  <si>
+    <t>Morning Shift B</t>
+  </si>
+  <si>
+    <t>Morning Shift C</t>
+  </si>
+  <si>
+    <t>Morning Shift D</t>
+  </si>
+  <si>
+    <t>Morning Shift E</t>
+  </si>
+  <si>
+    <t>Roster name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,13 +131,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -163,12 +171,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -187,9 +194,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -227,9 +234,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -262,26 +269,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -314,26 +304,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -508,25 +481,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -542,119 +514,119 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="2">
-        <v>1</v>
+      <c r="C2" t="s">
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2">
-        <v>2</v>
+      <c r="C3" t="s">
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="2">
-        <v>3</v>
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="2">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2">
         <v>15</v>
       </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>